<commit_message>
feat: Implement cursor-based pagination for lineage graph endpoints and update related API responses
</commit_message>
<xml_diff>
--- a/qlik_atlas_analytics_catalog.xlsx
+++ b/qlik_atlas_analytics_catalog.xlsx
@@ -2432,45 +2432,49 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Mittel</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Graph Pagination</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Voller In-Memory Load des Lineage-Graphen. Problematisch bei grossen Tenants.</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>backend/app/db_runtime_views.py</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Cursor-basierte Pagination empfohlen</t>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Cursor-basierte Pagination fuer Lineage-Graph. Keyset auf node_id, page_size 10-5000. Frontend auto-paginiert.</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>backend/shared/models.py, backend/app/runtime_query_rows.py, backend/app/db_runtime_views.py, backend/main.py, frontend/lineage.html</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Rueckwaertskompatibel: ohne page_size Parameter bleibt altes Verhalten</t>
         </is>
       </c>
     </row>

</xml_diff>